<commit_message>
coluna de preco opcional em modelo.xlsx
</commit_message>
<xml_diff>
--- a/modelo.xlsx
+++ b/modelo.xlsx
@@ -423,11 +423,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -441,6 +442,11 @@
           <t>QUANTIDADE</t>
         </is>
       </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>PRECO (opcional)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>